<commit_message>
feat(항구): WUHAN 신규 서비스 추가 (SNK 단독, N.CHINA 내륙)
- APP_POLS에 WUHAN 등록 (업로드 POL 인식)
- SNK_POL_EXPAND에 WUHAN / "WUHAN VIA SHA(BARGE)" 별칭 추가
- FR 운임표에 N.CHINA WUHAN 행 추가 (SNK 운임 시드, DY·CK 미서비스)
  · 실제 운임은 표준양식 엑셀 업로드로 덮어씀 (고객 화면은 업로드값만 노출)
- PM에 "Wuhan":"WUHAN" 매핑 — 렌탈(Wuhan)·해상 연동
- 표준양식 엑셀(SNK_rates_표준양식)에 WUHAN 행 추가 (노란색 강조)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lxz8bWkCunHFhXwYL3znTZ
</commit_message>
<xml_diff>
--- a/SNK_rates_표준양식.xlsx
+++ b/SNK_rates_표준양식.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +54,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -94,6 +99,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1076,49 +1085,49 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>S.CHINA</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>SHEKOU</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D14" s="5" t="n">
+          <t>N.CHINA</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
         <v>1700</v>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>1300</v>
-      </c>
-      <c r="F14" s="5" t="n">
+      <c r="D14" s="7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E14" s="7" t="n">
         <v>1650</v>
       </c>
-      <c r="G14" s="5" t="n">
-        <v>1450</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>1880</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>1400</v>
-      </c>
-      <c r="J14" s="5" t="n">
-        <v>1770</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>180</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>120</v>
+      <c r="F14" s="7" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1780</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>1730</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -1129,14 +1138,14 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>XIAMEN</t>
+          <t>SHEKOU</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
         <v>1350</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>1800</v>
+        <v>1700</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>1300</v>
@@ -1148,7 +1157,7 @@
         <v>1450</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>1950</v>
+        <v>1880</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>1400</v>
@@ -1160,7 +1169,7 @@
         <v>100</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>100</v>
@@ -1177,7 +1186,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>NANSHA</t>
+          <t>XIAMEN</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -1190,7 +1199,7 @@
         <v>1300</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>1450</v>
@@ -1202,7 +1211,7 @@
         <v>1400</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>1820</v>
+        <v>1770</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>100</v>
@@ -1214,7 +1223,7 @@
         <v>100</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17">
@@ -1225,27 +1234,45 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>YANTIAN</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n"/>
+          <t>NANSHA</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1350</v>
+      </c>
       <c r="D17" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>1950</v>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n">
-        <v>2050</v>
-      </c>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
+      <c r="I17" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>1820</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>100</v>
+      </c>
       <c r="L17" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
+        <v>150</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1255,45 +1282,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>HONGKONG</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>2400</v>
-      </c>
+          <t>YANTIAN</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n">
-        <v>2950</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>2300</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>2850</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>2500</v>
-      </c>
+        <v>1950</v>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>2400</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>3000</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>100</v>
-      </c>
+        <v>2050</v>
+      </c>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>150</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1303,32 +1312,32 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>SHANTOU</t>
+          <t>HONGKONG</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>1350</v>
+        <v>2400</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>1950</v>
+        <v>2950</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1300</v>
+        <v>2300</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1700</v>
+        <v>2850</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>2100</v>
+        <v>3100</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>1400</v>
+        <v>2400</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>1850</v>
+        <v>3000</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>100</v>
@@ -1351,7 +1360,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>HUANGPU/PRD</t>
+          <t>SHANTOU</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -1394,37 +1403,37 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>S.CHINA</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>JAPAN ALL PORTS</t>
+          <t>HUANGPU/PRD</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>1800</v>
+        <v>1950</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>1800</v>
+        <v>1700</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>1700</v>
+        <v>1450</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>1950</v>
+        <v>2100</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>1720</v>
+        <v>1400</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>2000</v>
+        <v>1850</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>100</v>
@@ -1433,46 +1442,46 @@
         <v>150</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM</t>
+          <t>JAPAN</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HOCHIMINH</t>
+          <t>JAPAN ALL PORTS</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>1100</v>
+        <v>1600</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>1450</v>
+        <v>1800</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>1800</v>
+        <v>1950</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>1200</v>
+        <v>1720</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>100</v>
@@ -1481,10 +1490,10 @@
         <v>150</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23">
@@ -1495,32 +1504,32 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HAIPHONG</t>
+          <t>HOCHIMINH</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>1200</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1750</v>
+        <v>1650</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>1100</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="G23" s="5" t="n">
         <v>1300</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>1200</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>100</v>
@@ -1532,7 +1541,7 @@
         <v>100</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24">
@@ -1543,32 +1552,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>DANANG</t>
+          <t>HAIPHONG</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>2100</v>
+        <v>1200</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>2750</v>
+        <v>1750</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>2000</v>
+        <v>1100</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>2550</v>
+        <v>1500</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>2200</v>
+        <v>1300</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>2900</v>
+        <v>1900</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>2100</v>
+        <v>1200</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>2700</v>
+        <v>1700</v>
       </c>
       <c r="K24" s="5" t="n">
         <v>100</v>
@@ -1580,55 +1589,55 @@
         <v>100</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>TAIWAN</t>
+          <t>VIETNAM</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>KEELUNG</t>
+          <t>DANANG</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>1500</v>
+        <v>2100</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1800</v>
+        <v>2750</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>1700</v>
+        <v>2550</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>1600</v>
+        <v>2200</v>
       </c>
       <c r="H25" s="5" t="n">
+        <v>2900</v>
+      </c>
+      <c r="I25" s="5" t="n">
         <v>2100</v>
       </c>
-      <c r="I25" s="5" t="n">
-        <v>1520</v>
-      </c>
       <c r="J25" s="5" t="n">
-        <v>1790</v>
+        <v>2700</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>100</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
@@ -1639,7 +1648,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KAOHSIUNG</t>
+          <t>KEELUNG</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
@@ -1687,35 +1696,35 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TAICHUNG</t>
+          <t>KAOHSIUNG</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D27" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="E27" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>2100</v>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>1920</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>2400</v>
-      </c>
       <c r="I27" s="5" t="n">
-        <v>1820</v>
+        <v>1520</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>2070</v>
+        <v>1790</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="L27" s="5" t="n">
         <v>300</v>
@@ -1724,55 +1733,55 @@
         <v>120</v>
       </c>
       <c r="N27" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>THAILAND</t>
+          <t>TAIWAN</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>BANGKOK</t>
+          <t>TAICHUNG</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>1400</v>
+        <v>1800</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>1850</v>
+        <v>2100</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1100</v>
+        <v>1700</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1500</v>
+        <v>1920</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>2000</v>
+        <v>2400</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1200</v>
+        <v>1820</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>1650</v>
+        <v>2070</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -1783,7 +1792,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>LAEM CHABANG</t>
+          <t>BANGKOK</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -1826,49 +1835,49 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>THAILAND</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>JAKARTA</t>
+          <t>LAEM CHABANG</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F30" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D30" s="5" t="n">
-        <v>1950</v>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>1750</v>
-      </c>
       <c r="G30" s="5" t="n">
-        <v>1620</v>
+        <v>1500</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>2130</v>
+        <v>2000</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>1520</v>
+        <v>1200</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>1930</v>
+        <v>1650</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31">
@@ -1879,11 +1888,11 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>SURABAYA</t>
+          <t>JAKARTA</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>1950</v>
@@ -1895,7 +1904,7 @@
         <v>1750</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>1460</v>
+        <v>1620</v>
       </c>
       <c r="H31" s="5" t="n">
         <v>2130</v>
@@ -1907,7 +1916,7 @@
         <v>1930</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="L31" s="5" t="n">
         <v>180</v>
@@ -1927,35 +1936,35 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>SEMARANG</t>
+          <t>SURABAYA</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>1800</v>
+        <v>1300</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>2350</v>
+        <v>1950</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>2150</v>
+        <v>1750</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>1920</v>
+        <v>1460</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>2530</v>
+        <v>2130</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>1820</v>
+        <v>1520</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>2330</v>
+        <v>1930</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="L32" s="5" t="n">
         <v>180</v>
@@ -1975,7 +1984,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>BELAWAN</t>
+          <t>SEMARANG</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -2023,7 +2032,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>PANJANG</t>
+          <t>BELAWAN</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -2071,7 +2080,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>MAKASSAR</t>
+          <t>PANJANG</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -2119,7 +2128,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>PALEMBANG</t>
+          <t>MAKASSAR</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -2162,49 +2171,49 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>OTHERS</t>
+          <t>INDONESIA</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
+          <t>PALEMBANG</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>2250</v>
+        <v>2350</v>
       </c>
       <c r="E37" s="5" t="n">
         <v>1700</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>2050</v>
+        <v>2150</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>1920</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>2400</v>
+        <v>2530</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>1820</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>2200</v>
+        <v>2330</v>
       </c>
       <c r="K37" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="M37" s="5" t="n">
         <v>120</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38">
@@ -2215,7 +2224,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>MANILA</t>
+          <t>SINGAPORE</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
@@ -2263,7 +2272,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>MALAYSIA (P.KLANG)</t>
+          <t>MANILA</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
@@ -2311,11 +2320,11 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>PASIR GUDANG</t>
+          <t>MALAYSIA (P.KLANG)</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2250</v>
@@ -2327,7 +2336,7 @@
         <v>2050</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>1750</v>
+        <v>1920</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>2400</v>
@@ -2339,7 +2348,7 @@
         <v>2200</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="L40" s="5" t="n">
         <v>150</v>
@@ -2359,7 +2368,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>PENANG</t>
+          <t>PASIR GUDANG</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -2407,11 +2416,11 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>TANJUNG PELEPAS</t>
+          <t>PENANG</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2250</v>
@@ -2423,7 +2432,7 @@
         <v>2050</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1920</v>
+        <v>1750</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>2400</v>
@@ -2435,7 +2444,7 @@
         <v>2200</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="L42" s="5" t="n">
         <v>150</v>
@@ -2455,44 +2464,44 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>CHATTOGRAM</t>
+          <t>TANJUNG PELEPAS</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>2250</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1800</v>
+        <v>1700</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>2150</v>
+        <v>2050</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2020</v>
+        <v>1920</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>2450</v>
+        <v>2400</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>1920</v>
+        <v>1820</v>
       </c>
       <c r="J43" s="5" t="n">
-        <v>2350</v>
+        <v>2200</v>
       </c>
       <c r="K43" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="M43" s="5" t="n">
         <v>120</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44">
@@ -2503,38 +2512,38 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>INDIA (MUNDRA)</t>
+          <t>CHATTOGRAM</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
-        <v>1800</v>
+        <v>1900</v>
       </c>
       <c r="D44" s="5" t="n">
         <v>2250</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>2250</v>
+        <v>2150</v>
       </c>
       <c r="G44" s="5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>2450</v>
+      </c>
+      <c r="I44" s="5" t="n">
         <v>1920</v>
       </c>
-      <c r="H44" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I44" s="5" t="n">
-        <v>1820</v>
-      </c>
       <c r="J44" s="5" t="n">
-        <v>2450</v>
+        <v>2350</v>
       </c>
       <c r="K44" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="M44" s="5" t="n">
         <v>120</v>
@@ -2551,7 +2560,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>NHAVA SHEVA</t>
+          <t>INDIA (MUNDRA)</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -2599,38 +2608,38 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>INDIA (CHENNAI)</t>
+          <t>NHAVA SHEVA</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
-        <v>2100</v>
+        <v>1800</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>2750</v>
+        <v>2250</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2000</v>
+        <v>1700</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>2550</v>
+        <v>2250</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>2220</v>
+        <v>1920</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>2950</v>
+        <v>2500</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>2120</v>
+        <v>1820</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>2750</v>
+        <v>2450</v>
       </c>
       <c r="K46" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="M46" s="5" t="n">
         <v>120</v>
@@ -2647,32 +2656,32 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>JEBEL ALI</t>
+          <t>INDIA (CHENNAI)</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
-        <v>2600</v>
+        <v>2100</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>3750</v>
+        <v>2750</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>3550</v>
+        <v>2550</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>2720</v>
+        <v>2220</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>3950</v>
+        <v>2950</v>
       </c>
       <c r="I47" s="5" t="n">
-        <v>2620</v>
+        <v>2120</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>3750</v>
+        <v>2750</v>
       </c>
       <c r="K47" s="5" t="n">
         <v>120</v>
@@ -2684,6 +2693,54 @@
         <v>120</v>
       </c>
       <c r="N47" s="5" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>OTHERS</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>JEBEL ALI</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>2720</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>3950</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>2620</v>
+      </c>
+      <c r="J48" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K48" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="L48" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="M48" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="N48" s="5" t="n">
         <v>200</v>
       </c>
     </row>
@@ -2703,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3318,49 +3375,49 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>S.CHINA</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>SHEKOU</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>1450</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>1900</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>1750</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>1600</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>2180</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>1550</v>
-      </c>
-      <c r="J14" s="5" t="n">
-        <v>2070</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>280</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>320</v>
+          <t>N.CHINA</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1780</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>1730</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>2300</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -3371,14 +3428,14 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>XIAMEN</t>
+          <t>SHEKOU</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
         <v>1450</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>1400</v>
@@ -3390,7 +3447,7 @@
         <v>1600</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>2250</v>
+        <v>2180</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>1550</v>
@@ -3402,7 +3459,7 @@
         <v>150</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>150</v>
@@ -3419,7 +3476,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>NANSHA</t>
+          <t>XIAMEN</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -3432,7 +3489,7 @@
         <v>1400</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>1700</v>
+        <v>1750</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>1600</v>
@@ -3444,7 +3501,7 @@
         <v>1550</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>2120</v>
+        <v>2070</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>150</v>
@@ -3456,7 +3513,7 @@
         <v>150</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>420</v>
+        <v>320</v>
       </c>
     </row>
     <row r="17">
@@ -3467,27 +3524,45 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>YANTIAN</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n"/>
+          <t>NANSHA</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1450</v>
+      </c>
       <c r="D17" s="5" t="n">
-        <v>2150</v>
-      </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
+        <v>2000</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>1600</v>
+      </c>
       <c r="H17" s="5" t="n">
-        <v>2450</v>
-      </c>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
+        <v>2250</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>1550</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>2120</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>150</v>
+      </c>
       <c r="L17" s="5" t="n">
-        <v>300</v>
-      </c>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
+        <v>250</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3497,45 +3572,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>HONGKONG</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>2500</v>
-      </c>
+          <t>YANTIAN</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n">
-        <v>3150</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>2400</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>2950</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>2650</v>
-      </c>
+        <v>2150</v>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n">
-        <v>3400</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>2550</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>3300</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>150</v>
-      </c>
+        <v>2450</v>
+      </c>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n">
-        <v>250</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>350</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -3545,32 +3602,32 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>SHANTOU</t>
+          <t>HONGKONG</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>1450</v>
+        <v>2500</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>2150</v>
+        <v>3150</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1400</v>
+        <v>2400</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>1800</v>
+        <v>2950</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>1600</v>
+        <v>2650</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>2400</v>
+        <v>3400</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>1550</v>
+        <v>2550</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>2150</v>
+        <v>3300</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>150</v>
@@ -3593,7 +3650,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>HUANGPU/PRD</t>
+          <t>SHANTOU</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -3636,85 +3693,85 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>S.CHINA</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>JAPAN ALL PORTS</t>
+          <t>HUANGPU/PRD</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>1600</v>
+        <v>1450</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>1800</v>
+        <v>2150</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>1950</v>
+        <v>2400</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>1720</v>
+        <v>1550</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>2000</v>
+        <v>2150</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>200</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM</t>
+          <t>JAPAN</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HOCHIMINH</t>
+          <t>JAPAN ALL PORTS</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>1200</v>
+        <v>1600</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>1650</v>
+        <v>1800</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>1100</v>
+        <v>1600</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>1450</v>
+        <v>1800</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>1800</v>
+        <v>1950</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>1200</v>
+        <v>1720</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>1600</v>
+        <v>2000</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>100</v>
@@ -3723,10 +3780,10 @@
         <v>150</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23">
@@ -3737,32 +3794,32 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HAIPHONG</t>
+          <t>HOCHIMINH</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>1200</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>1750</v>
+        <v>1650</v>
       </c>
       <c r="E23" s="5" t="n">
         <v>1100</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>1500</v>
+        <v>1450</v>
       </c>
       <c r="G23" s="5" t="n">
         <v>1300</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>1200</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>1700</v>
+        <v>1600</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>100</v>
@@ -3774,7 +3831,7 @@
         <v>100</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24">
@@ -3785,32 +3842,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>DANANG</t>
+          <t>HAIPHONG</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>2100</v>
+        <v>1200</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>2750</v>
+        <v>1750</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>2000</v>
+        <v>1100</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>2550</v>
+        <v>1500</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>2200</v>
+        <v>1300</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>2900</v>
+        <v>1900</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>2100</v>
+        <v>1200</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>2700</v>
+        <v>1700</v>
       </c>
       <c r="K24" s="5" t="n">
         <v>100</v>
@@ -3822,55 +3879,55 @@
         <v>100</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>TAIWAN</t>
+          <t>VIETNAM</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>KEELUNG</t>
+          <t>DANANG</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>1500</v>
+        <v>2100</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1800</v>
+        <v>2750</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>1700</v>
+        <v>2550</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>1600</v>
+        <v>2200</v>
       </c>
       <c r="H25" s="5" t="n">
+        <v>2900</v>
+      </c>
+      <c r="I25" s="5" t="n">
         <v>2100</v>
       </c>
-      <c r="I25" s="5" t="n">
-        <v>1520</v>
-      </c>
       <c r="J25" s="5" t="n">
-        <v>1790</v>
+        <v>2700</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>100</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
@@ -3881,7 +3938,7 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KAOHSIUNG</t>
+          <t>KEELUNG</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
@@ -3929,35 +3986,35 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TAICHUNG</t>
+          <t>KAOHSIUNG</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D27" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="E27" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <v>2100</v>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F27" s="5" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>1920</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>2400</v>
-      </c>
       <c r="I27" s="5" t="n">
-        <v>1820</v>
+        <v>1520</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>2070</v>
+        <v>1790</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="L27" s="5" t="n">
         <v>300</v>
@@ -3966,55 +4023,55 @@
         <v>120</v>
       </c>
       <c r="N27" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>THAILAND</t>
+          <t>TAIWAN</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>BANGKOK</t>
+          <t>TAICHUNG</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>1400</v>
+        <v>1800</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>1850</v>
+        <v>2100</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1100</v>
+        <v>1700</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1500</v>
+        <v>1920</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>2000</v>
+        <v>2400</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1200</v>
+        <v>1820</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>1650</v>
+        <v>2070</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -4025,7 +4082,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>LAEM CHABANG</t>
+          <t>BANGKOK</t>
         </is>
       </c>
       <c r="C29" s="5" t="n">
@@ -4068,49 +4125,49 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>THAILAND</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>JAKARTA</t>
+          <t>LAEM CHABANG</t>
         </is>
       </c>
       <c r="C30" s="5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F30" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="D30" s="5" t="n">
-        <v>1950</v>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>1400</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>1750</v>
-      </c>
       <c r="G30" s="5" t="n">
-        <v>1620</v>
+        <v>1500</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>2130</v>
+        <v>2000</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>1520</v>
+        <v>1200</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>1930</v>
+        <v>1650</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31">
@@ -4121,11 +4178,11 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>SURABAYA</t>
+          <t>JAKARTA</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
-        <v>1300</v>
+        <v>1500</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>1950</v>
@@ -4137,7 +4194,7 @@
         <v>1750</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>1460</v>
+        <v>1620</v>
       </c>
       <c r="H31" s="5" t="n">
         <v>2130</v>
@@ -4149,7 +4206,7 @@
         <v>1930</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="L31" s="5" t="n">
         <v>180</v>
@@ -4169,35 +4226,35 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>SEMARANG</t>
+          <t>SURABAYA</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>1800</v>
+        <v>1300</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>2350</v>
+        <v>1950</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>2150</v>
+        <v>1750</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>1920</v>
+        <v>1460</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>2530</v>
+        <v>2130</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>1820</v>
+        <v>1520</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>2330</v>
+        <v>1930</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="L32" s="5" t="n">
         <v>180</v>
@@ -4217,7 +4274,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>BELAWAN</t>
+          <t>SEMARANG</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
@@ -4265,7 +4322,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>PANJANG</t>
+          <t>BELAWAN</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
@@ -4313,7 +4370,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>MAKASSAR</t>
+          <t>PANJANG</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
@@ -4361,7 +4418,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>PALEMBANG</t>
+          <t>MAKASSAR</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
@@ -4404,49 +4461,49 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>OTHERS</t>
+          <t>INDONESIA</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
+          <t>PALEMBANG</t>
         </is>
       </c>
       <c r="C37" s="5" t="n">
         <v>1800</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>2250</v>
+        <v>2350</v>
       </c>
       <c r="E37" s="5" t="n">
         <v>1700</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>2050</v>
+        <v>2150</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>1920</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>2400</v>
+        <v>2530</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>1820</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>2200</v>
+        <v>2330</v>
       </c>
       <c r="K37" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="M37" s="5" t="n">
         <v>120</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38">
@@ -4457,7 +4514,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>MANILA</t>
+          <t>SINGAPORE</t>
         </is>
       </c>
       <c r="C38" s="5" t="n">
@@ -4505,7 +4562,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>MALAYSIA (P.KLANG)</t>
+          <t>MANILA</t>
         </is>
       </c>
       <c r="C39" s="5" t="n">
@@ -4553,11 +4610,11 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>PASIR GUDANG</t>
+          <t>MALAYSIA (P.KLANG)</t>
         </is>
       </c>
       <c r="C40" s="5" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2250</v>
@@ -4569,7 +4626,7 @@
         <v>2050</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>1750</v>
+        <v>1920</v>
       </c>
       <c r="H40" s="5" t="n">
         <v>2400</v>
@@ -4581,7 +4638,7 @@
         <v>2200</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="L40" s="5" t="n">
         <v>150</v>
@@ -4601,7 +4658,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>PENANG</t>
+          <t>PASIR GUDANG</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
@@ -4649,11 +4706,11 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>TANJUNG PELEPAS</t>
+          <t>PENANG</t>
         </is>
       </c>
       <c r="C42" s="5" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2250</v>
@@ -4665,7 +4722,7 @@
         <v>2050</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1920</v>
+        <v>1750</v>
       </c>
       <c r="H42" s="5" t="n">
         <v>2400</v>
@@ -4677,7 +4734,7 @@
         <v>2200</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="L42" s="5" t="n">
         <v>150</v>
@@ -4697,44 +4754,44 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>CHATTOGRAM</t>
+          <t>TANJUNG PELEPAS</t>
         </is>
       </c>
       <c r="C43" s="5" t="n">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="D43" s="5" t="n">
         <v>2250</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1800</v>
+        <v>1700</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>2150</v>
+        <v>2050</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>2020</v>
+        <v>1920</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>2450</v>
+        <v>2400</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>1920</v>
+        <v>1820</v>
       </c>
       <c r="J43" s="5" t="n">
-        <v>2350</v>
+        <v>2200</v>
       </c>
       <c r="K43" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="M43" s="5" t="n">
         <v>120</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44">
@@ -4745,38 +4802,38 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>INDIA (MUNDRA)</t>
+          <t>CHATTOGRAM</t>
         </is>
       </c>
       <c r="C44" s="5" t="n">
-        <v>1800</v>
+        <v>1900</v>
       </c>
       <c r="D44" s="5" t="n">
         <v>2250</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1700</v>
+        <v>1800</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>2250</v>
+        <v>2150</v>
       </c>
       <c r="G44" s="5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>2450</v>
+      </c>
+      <c r="I44" s="5" t="n">
         <v>1920</v>
       </c>
-      <c r="H44" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I44" s="5" t="n">
-        <v>1820</v>
-      </c>
       <c r="J44" s="5" t="n">
-        <v>2450</v>
+        <v>2350</v>
       </c>
       <c r="K44" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="M44" s="5" t="n">
         <v>120</v>
@@ -4793,7 +4850,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>NHAVA SHEVA</t>
+          <t>INDIA (MUNDRA)</t>
         </is>
       </c>
       <c r="C45" s="5" t="n">
@@ -4841,38 +4898,38 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>INDIA (CHENNAI)</t>
+          <t>NHAVA SHEVA</t>
         </is>
       </c>
       <c r="C46" s="5" t="n">
-        <v>2100</v>
+        <v>1800</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>2750</v>
+        <v>2250</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2000</v>
+        <v>1700</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>2550</v>
+        <v>2250</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>2220</v>
+        <v>1920</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>2950</v>
+        <v>2500</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>2120</v>
+        <v>1820</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>2750</v>
+        <v>2450</v>
       </c>
       <c r="K46" s="5" t="n">
         <v>120</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="M46" s="5" t="n">
         <v>120</v>
@@ -4889,32 +4946,32 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>JEBEL ALI</t>
+          <t>INDIA (CHENNAI)</t>
         </is>
       </c>
       <c r="C47" s="5" t="n">
-        <v>2600</v>
+        <v>2100</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>3750</v>
+        <v>2750</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>3550</v>
+        <v>2550</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>2720</v>
+        <v>2220</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>3950</v>
+        <v>2950</v>
       </c>
       <c r="I47" s="5" t="n">
-        <v>2620</v>
+        <v>2120</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>3750</v>
+        <v>2750</v>
       </c>
       <c r="K47" s="5" t="n">
         <v>120</v>
@@ -4926,6 +4983,54 @@
         <v>120</v>
       </c>
       <c r="N47" s="5" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>OTHERS</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>JEBEL ALI</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E48" s="5" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>2720</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>3950</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>2620</v>
+      </c>
+      <c r="J48" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="K48" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="L48" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="M48" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="N48" s="5" t="n">
         <v>200</v>
       </c>
     </row>

</xml_diff>